<commit_message>
added results in r1 for EnvironmentWorkerGroupRelationServiceTest
</commit_message>
<xml_diff>
--- a/r1/gen/finalReport.xlsx
+++ b/r1/gen/finalReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\r1\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2FA2C6-4B05-45E2-A082-46AFF7F2C949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43418148-2465-4D90-AD67-218A92B7637A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="56">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -205,6 +205,9 @@
   </si>
   <si>
     <t>0.024183</t>
+  </si>
+  <si>
+    <t>0.018274</t>
   </si>
 </sst>
 </file>
@@ -688,6 +691,9 @@
       <c r="C3">
         <v>2</v>
       </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -700,6 +706,9 @@
       <c r="C4">
         <v>0</v>
       </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
       <c r="I4">
         <v>0</v>
       </c>
@@ -715,6 +724,9 @@
       <c r="C5">
         <v>0</v>
       </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -757,6 +769,9 @@
       <c r="C7">
         <v>2</v>
       </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -768,6 +783,9 @@
       <c r="C8">
         <v>0</v>
       </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -779,6 +797,9 @@
       <c r="C9">
         <v>0</v>
       </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -819,6 +840,9 @@
       <c r="C11">
         <v>1</v>
       </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -830,6 +854,9 @@
       <c r="C12">
         <v>0</v>
       </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -841,6 +868,9 @@
       <c r="C13">
         <v>0</v>
       </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -910,6 +940,9 @@
       <c r="C16">
         <v>1</v>
       </c>
+      <c r="D16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -921,6 +954,9 @@
       <c r="C17">
         <v>1</v>
       </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -932,6 +968,9 @@
       <c r="C18">
         <v>0</v>
       </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -943,6 +982,9 @@
       <c r="C19">
         <v>0</v>
       </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -954,6 +996,9 @@
       <c r="C20">
         <v>0</v>
       </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -965,7 +1010,9 @@
       <c r="C21" s="2">
         <v>26.515000000000001</v>
       </c>
-      <c r="D21" s="2"/>
+      <c r="D21" s="2">
+        <v>19.774000000000001</v>
+      </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1011,7 +1058,9 @@
       <c r="C23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="1"/>
+      <c r="D23" s="1" t="s">
+        <v>55</v>
+      </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -1026,6 +1075,9 @@
         <v>22</v>
       </c>
       <c r="C24" t="s">
+        <v>22</v>
+      </c>
+      <c r="D24" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added results in r1 for ProcessServiceTest
</commit_message>
<xml_diff>
--- a/r1/gen/finalReport.xlsx
+++ b/r1/gen/finalReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\r1\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43418148-2465-4D90-AD67-218A92B7637A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B23B3B-647E-40A7-9FB3-71A8BDE7F647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -208,6 +208,9 @@
   </si>
   <si>
     <t>0.018274</t>
+  </si>
+  <si>
+    <t>0.018484</t>
   </si>
 </sst>
 </file>
@@ -694,6 +697,9 @@
       <c r="D3">
         <v>1</v>
       </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -709,6 +715,9 @@
       <c r="D4">
         <v>0</v>
       </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
       <c r="I4">
         <v>0</v>
       </c>
@@ -727,6 +736,9 @@
       <c r="D5">
         <v>0</v>
       </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -772,6 +784,9 @@
       <c r="D7">
         <v>0</v>
       </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -786,6 +801,9 @@
       <c r="D8">
         <v>0</v>
       </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -800,6 +818,9 @@
       <c r="D9">
         <v>0</v>
       </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -843,6 +864,9 @@
       <c r="D11">
         <v>0</v>
       </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -857,6 +881,9 @@
       <c r="D12">
         <v>0</v>
       </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -871,6 +898,9 @@
       <c r="D13">
         <v>0</v>
       </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -943,6 +973,9 @@
       <c r="D16">
         <v>1</v>
       </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -957,6 +990,9 @@
       <c r="D17">
         <v>1</v>
       </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -971,6 +1007,9 @@
       <c r="D18">
         <v>0</v>
       </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -985,6 +1024,9 @@
       <c r="D19">
         <v>0</v>
       </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -999,6 +1041,9 @@
       <c r="D20">
         <v>0</v>
       </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1013,7 +1058,9 @@
       <c r="D21" s="2">
         <v>19.774000000000001</v>
       </c>
-      <c r="E21" s="2"/>
+      <c r="E21" s="2">
+        <v>17.774999999999999</v>
+      </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -1061,7 +1108,9 @@
       <c r="D23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="1"/>
+      <c r="E23" s="1" t="s">
+        <v>56</v>
+      </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
@@ -1078,6 +1127,9 @@
         <v>22</v>
       </c>
       <c r="D24" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added results in r1 for McpConfigurationTest
</commit_message>
<xml_diff>
--- a/r1/gen/finalReport.xlsx
+++ b/r1/gen/finalReport.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\r1\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1B23B3B-647E-40A7-9FB3-71A8BDE7F647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89B7EA38-E252-4461-AE64-05DC356A0576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
     <sheet name="TEST IDS" sheetId="3" r:id="rId2"/>
+    <sheet name="Compilation errors" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -211,6 +212,23 @@
   </si>
   <si>
     <t>0.018484</t>
+  </si>
+  <si>
+    <t>0.009354</t>
+  </si>
+  <si>
+    <t>yes</t>
+  </si>
+  <si>
+    <t>cannot find symbol
+symbol:   method assertEquals(int,int)
+location: class com.alibaba.nacos.ai.config.ControllerMethodsCache_Proxy</t>
+  </si>
+  <si>
+    <t>Test case</t>
+  </si>
+  <si>
+    <t>Error</t>
   </si>
 </sst>
 </file>
@@ -261,12 +279,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -700,6 +724,9 @@
       <c r="E3">
         <v>1</v>
       </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -718,6 +745,9 @@
       <c r="E4">
         <v>0</v>
       </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
       <c r="I4">
         <v>0</v>
       </c>
@@ -739,6 +769,9 @@
       <c r="E5">
         <v>0</v>
       </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -787,6 +820,9 @@
       <c r="E7">
         <v>0</v>
       </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -804,6 +840,9 @@
       <c r="E8">
         <v>0</v>
       </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -821,6 +860,9 @@
       <c r="E9">
         <v>0</v>
       </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -867,6 +909,9 @@
       <c r="E11">
         <v>0</v>
       </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -884,6 +929,9 @@
       <c r="E12">
         <v>0</v>
       </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -901,6 +949,9 @@
       <c r="E13">
         <v>0</v>
       </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -976,6 +1027,9 @@
       <c r="E16">
         <v>1</v>
       </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -993,6 +1047,9 @@
       <c r="E17">
         <v>1</v>
       </c>
+      <c r="G17">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1010,6 +1067,9 @@
       <c r="E18">
         <v>0</v>
       </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1027,6 +1087,9 @@
       <c r="E19">
         <v>0</v>
       </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1044,6 +1107,9 @@
       <c r="E20">
         <v>0</v>
       </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1062,7 +1128,9 @@
         <v>17.774999999999999</v>
       </c>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="G21" s="2">
+        <v>17.058</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
     </row>
@@ -1112,7 +1180,9 @@
         <v>56</v>
       </c>
       <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
+      <c r="G23" s="1" t="s">
+        <v>57</v>
+      </c>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
     </row>
@@ -1131,6 +1201,9 @@
       </c>
       <c r="E24" t="s">
         <v>22</v>
+      </c>
+      <c r="G24" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -1252,4 +1325,34 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74A72989-0EB4-4966-868F-3AABF8D193B9}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="77.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="str">
+        <f>'TEST IDS'!C7</f>
+        <v>N.2</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added results in r1 for AuthHeaderUtilTest
</commit_message>
<xml_diff>
--- a/r1/gen/finalReport.xlsx
+++ b/r1/gen/finalReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\r1\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E45609F1-0FAB-4AEF-BDD0-BDA7D4A6F141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FAD349-7E46-4476-A1A7-9899D5C9EFCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -229,6 +229,14 @@
   </si>
   <si>
     <t>Error</t>
+  </si>
+  <si>
+    <t>cannot find symbol
+symbol:   method assertFalse(boolean)
+location: class com.alibaba.nacos.auth.util.NacosAuthConfig_Proxy</t>
+  </si>
+  <si>
+    <t>0.014895</t>
   </si>
 </sst>
 </file>
@@ -279,7 +287,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -290,6 +298,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -727,6 +738,9 @@
       <c r="G3">
         <v>0</v>
       </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -772,6 +786,9 @@
       <c r="G5">
         <v>0</v>
       </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
       <c r="O5" s="2"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
@@ -823,6 +840,9 @@
       <c r="G7">
         <v>1</v>
       </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -843,6 +863,9 @@
       <c r="G8">
         <v>0</v>
       </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -863,6 +886,9 @@
       <c r="G9">
         <v>0</v>
       </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -912,6 +938,9 @@
       <c r="G11">
         <v>0</v>
       </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
@@ -932,6 +961,9 @@
       <c r="G12">
         <v>0</v>
       </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
@@ -952,6 +984,9 @@
       <c r="G13">
         <v>0</v>
       </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
@@ -1030,6 +1065,9 @@
       <c r="G16">
         <v>1</v>
       </c>
+      <c r="I16">
+        <v>2</v>
+      </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
@@ -1050,6 +1088,9 @@
       <c r="G17">
         <v>1</v>
       </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1070,6 +1111,9 @@
       <c r="G18">
         <v>0</v>
       </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
@@ -1090,6 +1134,9 @@
       <c r="G19">
         <v>0</v>
       </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
@@ -1110,6 +1157,9 @@
       <c r="G20">
         <v>1</v>
       </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
@@ -1132,7 +1182,9 @@
         <v>17.058</v>
       </c>
       <c r="H21" s="2"/>
-      <c r="I21" s="2"/>
+      <c r="I21" s="2">
+        <v>15.94</v>
+      </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
@@ -1184,7 +1236,9 @@
         <v>57</v>
       </c>
       <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+      <c r="I23" s="1" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1203,6 +1257,9 @@
         <v>22</v>
       </c>
       <c r="G24" t="s">
+        <v>58</v>
+      </c>
+      <c r="I24" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1329,7 +1386,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74A72989-0EB4-4966-868F-3AABF8D193B9}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="77.5703125" customWidth="1"/>
@@ -1352,6 +1409,15 @@
         <v>59</v>
       </c>
     </row>
+    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="str">
+        <f>'TEST IDS'!C9</f>
+        <v>N.4</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added results in r1 for NamingHttpClientManagerTest
</commit_message>
<xml_diff>
--- a/r1/gen/finalReport.xlsx
+++ b/r1/gen/finalReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\r1\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64FAD349-7E46-4476-A1A7-9899D5C9EFCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9907BD15-FD28-4729-9D1B-6BA91FB967E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="66">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -237,6 +237,16 @@
   </si>
   <si>
     <t>0.014895</t>
+  </si>
+  <si>
+    <t>Compilation failure: 
+/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,80] illegal start of type
+/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,82] ';' expected
+/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,127] illegal start of expression
+/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,126] not a statement</t>
+  </si>
+  <si>
+    <t>0.011980</t>
   </si>
 </sst>
 </file>
@@ -738,6 +748,9 @@
       <c r="G3">
         <v>0</v>
       </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
       <c r="I3">
         <v>1</v>
       </c>
@@ -762,6 +775,9 @@
       <c r="G4">
         <v>0</v>
       </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
       <c r="I4">
         <v>0</v>
       </c>
@@ -786,6 +802,9 @@
       <c r="G5">
         <v>0</v>
       </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
       <c r="I5">
         <v>0</v>
       </c>
@@ -840,6 +859,9 @@
       <c r="G7">
         <v>1</v>
       </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
       <c r="I7">
         <v>1</v>
       </c>
@@ -863,6 +885,9 @@
       <c r="G8">
         <v>0</v>
       </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
       <c r="I8">
         <v>0</v>
       </c>
@@ -886,6 +911,9 @@
       <c r="G9">
         <v>0</v>
       </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
       <c r="I9">
         <v>0</v>
       </c>
@@ -938,6 +966,9 @@
       <c r="G11">
         <v>0</v>
       </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
       <c r="I11">
         <v>0</v>
       </c>
@@ -961,6 +992,9 @@
       <c r="G12">
         <v>0</v>
       </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
       <c r="I12">
         <v>0</v>
       </c>
@@ -984,6 +1018,9 @@
       <c r="G13">
         <v>0</v>
       </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
       <c r="I13">
         <v>0</v>
       </c>
@@ -1065,6 +1102,9 @@
       <c r="G16">
         <v>1</v>
       </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
       <c r="I16">
         <v>2</v>
       </c>
@@ -1088,6 +1128,9 @@
       <c r="G17">
         <v>1</v>
       </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
       <c r="I17">
         <v>2</v>
       </c>
@@ -1111,6 +1154,9 @@
       <c r="G18">
         <v>0</v>
       </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
       <c r="I18">
         <v>0</v>
       </c>
@@ -1134,6 +1180,9 @@
       <c r="G19">
         <v>0</v>
       </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
       <c r="I19">
         <v>0</v>
       </c>
@@ -1157,6 +1206,9 @@
       <c r="G20">
         <v>1</v>
       </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
       <c r="I20">
         <v>1</v>
       </c>
@@ -1181,7 +1233,9 @@
       <c r="G21" s="2">
         <v>17.058</v>
       </c>
-      <c r="H21" s="2"/>
+      <c r="H21" s="2">
+        <v>26.428999999999998</v>
+      </c>
       <c r="I21" s="2">
         <v>15.94</v>
       </c>
@@ -1235,7 +1289,9 @@
       <c r="G23" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="H23" s="1"/>
+      <c r="H23" s="1" t="s">
+        <v>65</v>
+      </c>
       <c r="I23" s="1" t="s">
         <v>63</v>
       </c>
@@ -1257,6 +1313,9 @@
         <v>22</v>
       </c>
       <c r="G24" t="s">
+        <v>58</v>
+      </c>
+      <c r="H24" t="s">
         <v>58</v>
       </c>
       <c r="I24" t="s">
@@ -1386,7 +1445,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74A72989-0EB4-4966-868F-3AABF8D193B9}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="77.5703125" customWidth="1"/>
@@ -1409,12 +1468,21 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="195" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="str">
+        <f>'TEST IDS'!C8</f>
+        <v>N.3</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="str">
         <f>'TEST IDS'!C9</f>
         <v>N.4</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B4" s="7" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added results in r1 for DefaultNamingSelectorTest
</commit_message>
<xml_diff>
--- a/r1/gen/finalReport.xlsx
+++ b/r1/gen/finalReport.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\r1\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9907BD15-FD28-4729-9D1B-6BA91FB967E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDAC756-C38D-4F51-BA2F-DF92590B4286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
-    <sheet name="TEST IDS" sheetId="3" r:id="rId2"/>
+    <sheet name="Test IDs" sheetId="3" r:id="rId2"/>
     <sheet name="Compilation errors" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="72">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -127,9 +127,6 @@
     <t>testShutdown</t>
   </si>
   <si>
-    <t>Needs human refactor</t>
-  </si>
-  <si>
     <t>TEST CLASS</t>
   </si>
   <si>
@@ -220,33 +217,46 @@
     <t>yes</t>
   </si>
   <si>
-    <t>cannot find symbol
-symbol:   method assertEquals(int,int)
-location: class com.alibaba.nacos.ai.config.ControllerMethodsCache_Proxy</t>
-  </si>
-  <si>
     <t>Test case</t>
   </si>
   <si>
-    <t>Error</t>
-  </si>
-  <si>
-    <t>cannot find symbol
-symbol:   method assertFalse(boolean)
-location: class com.alibaba.nacos.auth.util.NacosAuthConfig_Proxy</t>
-  </si>
-  <si>
     <t>0.014895</t>
   </si>
   <si>
-    <t>Compilation failure: 
-/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,80] illegal start of type
-/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,82] ';' expected
-/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,127] illegal start of expression
-/C:/Users/fedev/Documents/UNICAM/Phd/nacos/client/src/test/java/com/alibaba/nacos/client/naming/remote/http/NamingHttpClientManagerIntegrationTest_testShutdown.java:[21,126] not a statement</t>
-  </si>
-  <si>
     <t>0.011980</t>
+  </si>
+  <si>
+    <t>Junit import</t>
+  </si>
+  <si>
+    <t xml:space="preserve">configuration point </t>
+  </si>
+  <si>
+    <t>ControllerMethodsCache_Proxy</t>
+  </si>
+  <si>
+    <t>NamingHttpClientManagerIntegrationTest_testShutdown.java</t>
+  </si>
+  <si>
+    <t>NacosAuthConfig_Proxy</t>
+  </si>
+  <si>
+    <t>DefaultNamingSelectorIntegrationTest_testSelect</t>
+  </si>
+  <si>
+    <t>Error locations</t>
+  </si>
+  <si>
+    <t>Error types</t>
+  </si>
+  <si>
+    <t>Junit import, configuration point</t>
+  </si>
+  <si>
+    <t>Needs human refactor (see Compilation errors for details)</t>
+  </si>
+  <si>
+    <t>0.012227</t>
   </si>
 </sst>
 </file>
@@ -307,10 +317,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -664,38 +674,38 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" t="str">
-        <f>'TEST IDS'!C2</f>
+        <f>'Test IDs'!C2</f>
         <v>DS.1</v>
       </c>
       <c r="C1" t="str">
-        <f>'TEST IDS'!C3</f>
+        <f>'Test IDs'!C3</f>
         <v>DS.2</v>
       </c>
       <c r="D1" t="str">
-        <f>'TEST IDS'!C4</f>
+        <f>'Test IDs'!C4</f>
         <v>DS.3</v>
       </c>
       <c r="E1" t="str">
-        <f>'TEST IDS'!C5</f>
+        <f>'Test IDs'!C5</f>
         <v>DS.4</v>
       </c>
       <c r="F1" t="str">
-        <f>'TEST IDS'!C6</f>
+        <f>'Test IDs'!C6</f>
         <v>N.1</v>
       </c>
       <c r="G1" t="str">
-        <f>'TEST IDS'!C7</f>
+        <f>'Test IDs'!C7</f>
         <v>N.2</v>
       </c>
       <c r="H1" t="str">
-        <f>'TEST IDS'!C8</f>
+        <f>'Test IDs'!C8</f>
         <v>N.3</v>
       </c>
       <c r="I1" t="str">
-        <f>'TEST IDS'!C9</f>
+        <f>'Test IDs'!C9</f>
         <v>N.4</v>
       </c>
     </row>
@@ -745,6 +755,9 @@
       <c r="E3">
         <v>1</v>
       </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
       <c r="G3">
         <v>0</v>
       </c>
@@ -758,7 +771,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -770,6 +783,9 @@
         <v>0</v>
       </c>
       <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
@@ -785,7 +801,7 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -797,6 +813,9 @@
         <v>0</v>
       </c>
       <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
         <v>0</v>
       </c>
       <c r="G5">
@@ -856,6 +875,9 @@
       <c r="E7">
         <v>0</v>
       </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
       <c r="G7">
         <v>1</v>
       </c>
@@ -868,7 +890,7 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -880,6 +902,9 @@
         <v>0</v>
       </c>
       <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
@@ -894,7 +919,7 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -906,6 +931,9 @@
         <v>0</v>
       </c>
       <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
         <v>0</v>
       </c>
       <c r="G9">
@@ -920,7 +948,7 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -949,7 +977,7 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -961,6 +989,9 @@
         <v>0</v>
       </c>
       <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
         <v>0</v>
       </c>
       <c r="G11">
@@ -975,7 +1006,7 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -987,6 +1018,9 @@
         <v>0</v>
       </c>
       <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
         <v>0</v>
       </c>
       <c r="G12">
@@ -1001,7 +1035,7 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -1013,6 +1047,9 @@
         <v>0</v>
       </c>
       <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
         <v>0</v>
       </c>
       <c r="G13">
@@ -1027,7 +1064,7 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -1056,7 +1093,7 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1099,6 +1136,9 @@
       <c r="E16">
         <v>1</v>
       </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
       <c r="G16">
         <v>1</v>
       </c>
@@ -1125,6 +1165,9 @@
       <c r="E17">
         <v>1</v>
       </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
       <c r="G17">
         <v>1</v>
       </c>
@@ -1151,6 +1194,9 @@
       <c r="E18">
         <v>0</v>
       </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
       <c r="G18">
         <v>0</v>
       </c>
@@ -1177,6 +1223,9 @@
       <c r="E19">
         <v>0</v>
       </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
       <c r="G19">
         <v>0</v>
       </c>
@@ -1203,6 +1252,9 @@
       <c r="E20">
         <v>0</v>
       </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
       <c r="G20">
         <v>1</v>
       </c>
@@ -1229,7 +1281,9 @@
       <c r="E21" s="2">
         <v>17.774999999999999</v>
       </c>
-      <c r="F21" s="2"/>
+      <c r="F21" s="2">
+        <v>11.945</v>
+      </c>
       <c r="G21" s="2">
         <v>17.058</v>
       </c>
@@ -1274,31 +1328,33 @@
         <v>9</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="E23" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="F23" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="H23" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s">
         <v>22</v>
@@ -1312,14 +1368,17 @@
       <c r="E24" t="s">
         <v>22</v>
       </c>
+      <c r="F24" t="s">
+        <v>57</v>
+      </c>
       <c r="G24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1340,13 +1399,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1357,7 +1416,7 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1368,7 +1427,7 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1379,7 +1438,7 @@
         <v>15</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1390,7 +1449,7 @@
         <v>19</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1401,7 +1460,7 @@
         <v>21</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1412,7 +1471,7 @@
         <v>25</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1423,18 +1482,18 @@
         <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>48</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1445,45 +1504,70 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74A72989-0EB4-4966-868F-3AABF8D193B9}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="77.5703125" customWidth="1"/>
+    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>'Test IDs'!C6</f>
+        <v>N.1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="str">
+        <f>'Test IDs'!C7</f>
+        <v>N.2</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="C3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="str">
-        <f>'TEST IDS'!C7</f>
-        <v>N.2</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="195" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="str">
-        <f>'TEST IDS'!C8</f>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="str">
+        <f>'Test IDs'!C8</f>
         <v>N.3</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="str">
-        <f>'TEST IDS'!C9</f>
+      <c r="C4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="str">
+        <f>'Test IDs'!C9</f>
         <v>N.4</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>62</v>
+      <c r="B5" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>